<commit_message>
harvest(AD): add 3 new ⏳ Pending candidates — journal harvest 2026-10-11
New papers staged this week:
1. Anchor and Adapt (arXiv 2610.07016, Oct 4, 2026) — few-shot VLM/CLIP
   prompt adaptation, MVTec AD + VisA; added to 總覽, MVTec AD, VisA
2. VAND 4.0 Challenge Report (arXiv 2610.04392, Oct 3, 2026) — CVPR 2026
   benchmark report; MVTec AD 2 (SegF1) + Kaputt 2; added to 總覽, MVTec AD2
3. IndusAgent (arXiv 2605.20682, May 2026) — open-vocabulary zero-shot
   VLM/agentic, MVTec AD + VisA + MPDD; previously missed; added to 總覽,
   MVTec AD (already present), VisA, MPDD

All entries ⏳ Pending — arXiv HTML blocked, no GitHub repos found.
Email skipped (no .env SMTP credentials present).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012eMYhCgyd5eHf1AijkNyKz
</commit_message>
<xml_diff>
--- a/AnomalyDetection_Papers_Summary_v10_20260425.xlsx
+++ b/AnomalyDetection_Papers_Summary_v10_20260425.xlsx
@@ -1133,7 +1133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O266"/>
+  <dimension ref="A1:O269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="12" customWidth="1" style="27" min="1" max="1"/>
@@ -18486,6 +18486,152 @@
       <c r="N266" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2609.04775</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>MVTec AD, VisA (few-shot cross-dataset protocol; NON-STANDARD PROTOCOL)</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>基於視覺語言模型 (VLM-based) / CLIP / 非對稱提示自適應 (Asymmetric Prompt Adaptation) / 少樣本 (Few-Shot)</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Anchor and Adapt (Asymmetric Prompt Adaptation for Few-Shot Industrial Anomaly Detection)</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Mengyang Zhao, Teng Fu, Haiyang Yu, Ke Niu, Bin Li, Xiangyang Xue</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>arXiv 2610.07016 (2026-10-04)</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>⏳ Pending</t>
+        </is>
+      </c>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>⏳ Pending — arXiv 2610.07016 (Oct 4, 2026); arXiv HTML blocked, no GitHub repo found. Two-stage prompt learning framework: Stage I learns transferable normal/abnormal text anchors from annotated auxiliary data; Stage II freezes anchors and adapts an additional normal branch using few target normal images. Text-anchor regularization keeps adapted prompts consistent with generic normal prior and separated from abnormal anchors. Evaluates cross-dataset transfer in both directions between MVTec AD and VisA under 1-, 2-shot settings. Competes with PromptAD and template-based prompt methods. NON-STANDARD PROTOCOL (few-shot). Journal harvest 2026-10-11. [基於VLM/CLIP / 非對稱提示自適應 / 少樣本]</t>
+        </is>
+      </c>
+      <c r="N267" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2610.07016</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>MVTec AD 2, Kaputt 2 (VAND 4.0 Challenge benchmark report; CVPR 2026 workshop)</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>基準/挑戰賽報告 (Benchmark / Challenge Report) — MVTec AD 2 工業缺陷分割 + Kaputt 2 零售物流</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>VAND 4.0 Challenge Report (Detecting Defects that Matter: An Application-Driven Benchmark)</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>MVTec, TUM, Amazon, Intel, NVIDIA (VAND 4.0 organizing committee)</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>CVPR 2026 VAND 4.0 Workshop / arXiv 2610.04392 (2026-10-03)</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>⏳ Pending</t>
+        </is>
+      </c>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>⏳ Pending — arXiv 2610.04392 (Oct 3, 2026); CVPR 2026 VAND 4.0 Workshop challenge report. Industrial Track: MVTec AD 2, scored by pixel-level SegF1 (NOT AUROC). Regular setting: 9 submissions; best ~57% SegF1. Zero-shot: 5 submissions; trails by ~15 SegF1 pts. DINOv3 backbones dominate. Robustness to distribution shift flagged as open problem. Retail Track: Kaputt 2, scored by AP_any; supervised near-saturation for common defects; rare defect performance collapses (spillage ~53 AP, missing units ~27 AP). NOT a method paper — catalog reference entry. Journal harvest 2026-10-11. [基準/挑戰賽報告]</t>
+        </is>
+      </c>
+      <c r="N268" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2610.04392</t>
+        </is>
+      </c>
+      <c r="O268" t="inlineStr">
+        <is>
+          <t>https://github.com/cvpr-vand/vand-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>MVTec AD, VisA, MPDD, DTD, SDD (零樣本開放詞彙協議; NON-STANDARD PROTOCOL — open-vocabulary zero-shot)</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>基於基礎模型 (Foundation Model-based) / VLM / 代理工具增強 (Agentic Tools) / 開放詞彙 (Open-Vocabulary) / 零樣本</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>IndusAgent (Reinforcing Open-Vocabulary Industrial Anomaly Detection with Agentic Tools)</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Rongbin Tan, Huawei Cao, Shuhan Song et al. (13 authors)</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>arXiv 2605.20682 (2026-05-20)</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>⏳ Pending</t>
+        </is>
+      </c>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>⏳ Pending — arXiv 2605.20682 (May 20, 2026); arXiv HTML blocked, no GitHub found. Tool-augmented agentic framework for open-vocabulary IAD. Fine-tuned on custom Indus-CoT dataset with gated reinforcement learning objective (classification + localization + anomaly reasoning + tool usage). Uses dynamic region cropping, high-frequency feature enhancement, prior retrieval. Evaluates: MVTec-AD, VisA, MPDD, DTD, SDD — zero-shot protocol. Headline: avg score 83.4% (metric unclear from web snippet; NOT verified). NON-STANDARD PROTOCOL (open-vocabulary zero-shot). Previously missed in Aug/Sep harvests. Journal harvest 2026-10-11. [基於基礎模型/VLM / 代理工具增強 / 開放詞彙 / 零樣本]</t>
+        </is>
+      </c>
+      <c r="N269" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.20682</t>
         </is>
       </c>
     </row>
@@ -18698,7 +18844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O146"/>
+  <dimension ref="A1:O147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="12" customWidth="1" style="27" min="1" max="1"/>
@@ -28287,6 +28433,53 @@
       <c r="N146" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2609.04775</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>MVTec AD (few-shot cross-dataset protocol; NON-STANDARD PROTOCOL)</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>基於視覺語言模型 (VLM-based) / CLIP / 非對稱提示自適應 / 少樣本 (Few-Shot)</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Anchor and Adapt (Asymmetric Prompt Adaptation for Few-Shot Industrial Anomaly Detection)</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Mengyang Zhao, Teng Fu, Haiyang Yu, Ke Niu, Bin Li, Xiangyang Xue</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>arXiv 2610.07016 (2026-10-04)</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>⏳ Pending</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>⏳ Pending — few-shot cross-dataset protocol. arXiv HTML blocked; metrics not accessible. [基於VLM/CLIP / 非對稱提示自適應 / 少樣本]</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2610.07016</t>
         </is>
       </c>
     </row>
@@ -30180,7 +30373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:O20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="12" customWidth="1" style="27" min="1" max="1"/>
@@ -31486,6 +31679,58 @@
       <c r="O19" t="inlineStr">
         <is>
           <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>MVTec AD 2 (VAND 4.0 Challenge; pixel-level SegF1 metric — NOT AUROC)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>基準/挑戰賽報告 (Benchmark / Challenge Report)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>VAND 4.0 Challenge Report (Detecting Defects that Matter: Application-Driven Benchmark)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MVTec, TUM, Amazon, Intel, NVIDIA (VAND 4.0 organizing committee)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>CVPR 2026 VAND 4.0 Workshop / arXiv 2610.04392 (2026-10-03)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>⏳ Pending</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>⏳ Pending — benchmark/challenge report. MVTec AD 2 Industrial Track. Primary metric: pixel-level SegF1 (NOT AUROC). Best regular-setting entry: ~57% SegF1. Zero-shot entries trail by ~15 SegF1 pts. DINOv3 backbones dominate. Full leaderboard on benchmark.mvtec.com. NOT a standalone method paper. [基準/挑戰賽報告]</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2610.04392</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>https://github.com/cvpr-vand/vand-2026</t>
         </is>
       </c>
     </row>
@@ -31525,7 +31770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O100"/>
+  <dimension ref="A1:O102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="12" customWidth="1" style="27" min="1" max="1"/>
@@ -37959,6 +38204,100 @@
       <c r="N100" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2609.13282</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>VisA (few-shot cross-dataset protocol; NON-STANDARD PROTOCOL)</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>基於視覺語言模型 (VLM-based) / CLIP / 非對稱提示自適應 / 少樣本 (Few-Shot)</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Anchor and Adapt (Asymmetric Prompt Adaptation for Few-Shot Industrial Anomaly Detection)</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Mengyang Zhao, Teng Fu, Haiyang Yu, Ke Niu, Bin Li, Xiangyang Xue</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>arXiv 2610.07016 (2026-10-04)</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>⏳ Pending</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>⏳ Pending — few-shot cross-dataset protocol. arXiv HTML blocked; metrics not accessible. [基於VLM/CLIP / 非對稱提示自適應 / 少樣本]</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2610.07016</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>VisA (零樣本開放詞彙協議; NON-STANDARD PROTOCOL — open-vocabulary zero-shot)</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>基於基礎模型 (Foundation Model-based) / VLM / 代理工具增強 (Agentic Tools) / 開放詞彙 / 零樣本</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>IndusAgent (Reinforcing Open-Vocabulary Industrial Anomaly Detection with Agentic Tools)</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Rongbin Tan, Huawei Cao, Shuhan Song et al.</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>arXiv 2605.20682 (2026-05-20)</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>⏳ Pending</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>⏳ Pending — open-vocabulary zero-shot protocol. arXiv HTML blocked; metrics not accessible. [基於基礎模型/VLM / 代理 / 零樣本]</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.20682</t>
         </is>
       </c>
     </row>
@@ -38060,7 +38399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O25"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="12" customWidth="1" style="27" min="1" max="1"/>
@@ -39626,6 +39965,53 @@
       <c r="O25" t="inlineStr">
         <is>
           <t>https://github.com/Mingxiu-Cai/XMatchAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MPDD (零樣本開放詞彙協議; NON-STANDARD PROTOCOL — open-vocabulary zero-shot)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>基於基礎模型 (Foundation Model-based) / VLM / 代理工具增強 (Agentic Tools) / 開放詞彙 / 零樣本</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>IndusAgent (Reinforcing Open-Vocabulary Industrial Anomaly Detection with Agentic Tools)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Rongbin Tan, Huawei Cao, Shuhan Song et al.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>arXiv 2605.20682 (2026-05-20)</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>⏳ Pending</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>⏳ Pending — open-vocabulary zero-shot protocol. arXiv HTML blocked; metrics not accessible. [基於基礎模型/VLM / 代理 / 零樣本]</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.20682</t>
         </is>
       </c>
     </row>

</xml_diff>